<commit_message>
update to redox ED
</commit_message>
<xml_diff>
--- a/exposan/VFA/LCA data/impact_items.xlsx
+++ b/exposan/VFA/LCA data/impact_items.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/blues/Documents/EXPOsan/exposan/VFA/LCA data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A07EC946-CAB6-1343-B9D7-1B83E1D69F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CE9076-CCF3-824B-A124-B33E9345F955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32520" yWindow="-1540" windowWidth="29400" windowHeight="16760" activeTab="1" xr2:uid="{BD97E243-0BB4-3F42-9EBC-00D49E7EE019}"/>
+    <workbookView xWindow="32440" yWindow="-1980" windowWidth="29400" windowHeight="16760" activeTab="1" xr2:uid="{BD97E243-0BB4-3F42-9EBC-00D49E7EE019}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="33">
   <si>
     <t>uniform</t>
   </si>
@@ -76,9 +76,6 @@
     <t>m</t>
   </si>
   <si>
-    <t>ecoinvent 3.8 - cutoff, TRACI</t>
-  </si>
-  <si>
     <t>Aluminum</t>
   </si>
   <si>
@@ -107,6 +104,36 @@
   </si>
   <si>
     <t>area?</t>
+  </si>
+  <si>
+    <t>ecoinvent 3.11 - cutoff, TRACI v2.1 LT</t>
+  </si>
+  <si>
+    <t>StainlessSteel</t>
+  </si>
+  <si>
+    <t>TiElectrode</t>
+  </si>
+  <si>
+    <t>AcrylicHousing</t>
+  </si>
+  <si>
+    <t>RedoxCouple</t>
+  </si>
+  <si>
+    <t>ElectricMotor</t>
+  </si>
+  <si>
+    <t>Hdpe</t>
+  </si>
+  <si>
+    <t>AugerConveyor</t>
+  </si>
+  <si>
+    <t>MembraneModule</t>
+  </si>
+  <si>
+    <t>PvcPiping</t>
   </si>
 </sst>
 </file>
@@ -143,24 +170,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -175,12 +190,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +525,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -520,7 +533,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
@@ -528,7 +541,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -536,15 +549,15 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -552,7 +565,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
         <v>12</v>
@@ -568,7 +581,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -582,7 +595,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B26" t="s">
         <v>8</v>
@@ -590,7 +603,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" t="s">
         <v>8</v>
@@ -603,7 +616,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28627DAA-889C-6942-A3B5-3C8A993554C1}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
@@ -636,252 +649,294 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
       </c>
       <c r="C2">
-        <v>54</v>
+        <v>24.4</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D9" si="0">C2*0.9</f>
-        <v>48.6</v>
+        <f t="shared" ref="D2:D7" si="0">C2*0.9</f>
+        <v>21.96</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E9" si="1">C2*1.1</f>
-        <v>59.400000000000006</v>
+        <f t="shared" ref="E2:E7" si="1">C2*1.1</f>
+        <v>26.84</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
         <v>11</v>
       </c>
       <c r="C3">
-        <v>0.11600000000000001</v>
+        <v>46.1</v>
       </c>
       <c r="D3">
         <f t="shared" si="0"/>
-        <v>0.10440000000000001</v>
+        <v>41.49</v>
       </c>
       <c r="E3">
         <f t="shared" si="1"/>
-        <v>0.12760000000000002</v>
+        <v>50.710000000000008</v>
       </c>
       <c r="F3" t="s">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4">
-        <v>3.06</v>
+        <v>2.89</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>2.754</v>
+        <v>2.601</v>
       </c>
       <c r="E4">
         <f t="shared" si="1"/>
-        <v>3.3660000000000005</v>
+        <v>3.1790000000000003</v>
       </c>
       <c r="F4" t="s">
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>20</v>
+      <c r="A5" t="s">
+        <v>19</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5">
-        <v>8.2361676999999993</v>
+        <v>6.4073333333333347</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>7.4125509299999992</v>
+        <v>5.7666000000000013</v>
       </c>
       <c r="E5">
         <f t="shared" si="1"/>
-        <v>9.0597844700000003</v>
+        <v>7.0480666666666689</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
       <c r="C6">
-        <v>2.1800000000000002</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>1.9620000000000002</v>
+        <v>2.2410000000000001</v>
       </c>
       <c r="E6">
         <f t="shared" si="1"/>
-        <v>2.3980000000000006</v>
+        <v>2.7390000000000003</v>
       </c>
       <c r="F6" t="s">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
       </c>
       <c r="C7">
-        <v>1.06</v>
+        <v>1.25</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>0.95400000000000007</v>
+        <v>1.125</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
-        <v>1.1660000000000001</v>
+        <v>1.375</v>
       </c>
       <c r="F7" t="s">
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>1</v>
+      <c r="A8" t="s">
+        <v>24</v>
       </c>
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8">
-        <v>4.79</v>
+        <v>4.57</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
-        <v>4.3109999999999999</v>
+        <v>3.1989999999999998</v>
       </c>
       <c r="E8">
-        <f t="shared" si="1"/>
-        <v>5.2690000000000001</v>
+        <v>5.9410000000000007</v>
       </c>
       <c r="F8" t="s">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>14</v>
+      <c r="A9" t="s">
+        <v>27</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9">
-        <v>5.4695463000000002</v>
+        <v>4.57</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
-        <v>4.9225916700000001</v>
+        <f t="shared" ref="D9" si="2">C9*0.9</f>
+        <v>4.1130000000000004</v>
       </c>
       <c r="E9">
-        <f t="shared" si="1"/>
-        <v>6.0165009300000003</v>
+        <f t="shared" ref="E9" si="3">C9*1.1</f>
+        <v>5.027000000000001</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>15</v>
+      <c r="A10" t="s">
+        <v>29</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
       </c>
       <c r="C10">
-        <v>3.0634122000000001</v>
+        <v>2.75</v>
       </c>
       <c r="D10">
-        <f t="shared" ref="D10" si="2">C10*0.9</f>
-        <v>2.7570709800000004</v>
+        <f t="shared" ref="D10" si="4">C10*0.9</f>
+        <v>2.4750000000000001</v>
       </c>
       <c r="E10">
-        <f t="shared" ref="E10" si="3">C10*1.1</f>
-        <v>3.3697534200000003</v>
+        <f t="shared" ref="E10" si="5">C10*1.1</f>
+        <v>3.0250000000000004</v>
       </c>
       <c r="F10" t="s">
         <v>0</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>16</v>
+      <c r="A11" t="s">
+        <v>28</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11">
-        <v>6.5752404999999996</v>
+        <v>5685</v>
       </c>
       <c r="D11">
-        <f t="shared" ref="D11" si="4">C11*0.9</f>
-        <v>5.9177164499999995</v>
+        <v>4548</v>
       </c>
       <c r="E11">
-        <f t="shared" ref="E11" si="5">C11*1.1</f>
-        <v>7.2327645499999997</v>
+        <v>6822</v>
       </c>
       <c r="F11" t="s">
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>1400</v>
+      </c>
+      <c r="D12">
+        <v>979.99999999999989</v>
+      </c>
+      <c r="E12">
+        <v>1820</v>
+      </c>
+      <c r="F12" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>232</v>
+      </c>
+      <c r="D13">
+        <v>162.39999999999998</v>
+      </c>
+      <c r="E13">
+        <v>301.60000000000002</v>
+      </c>
+      <c r="F13" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>